<commit_message>
Complete lounge eligibility lookup table and justification
</commit_message>
<xml_diff>
--- a/Lounge Eligibility Lookup Template - Task 1.xlsx
+++ b/Lounge Eligibility Lookup Template - Task 1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\JDodson\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jerly\worky\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0229EC04-CD23-412F-956E-F8EE5E086E89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D221DF59-46C9-4371-A515-1485738AD8B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-90" yWindow="-90" windowWidth="19380" windowHeight="11460" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2660" yWindow="2660" windowWidth="14400" windowHeight="8170" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Lounge Eligibility Lookup Table" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="32">
   <si>
     <t>Grouping</t>
   </si>
@@ -41,9 +41,6 @@
     <t>Notes</t>
   </si>
   <si>
-    <t>Lounge Eligibility Lookup</t>
-  </si>
-  <si>
     <t>Prompt</t>
   </si>
   <si>
@@ -63,12 +60,72 @@
   </si>
   <si>
     <t>Justification:</t>
+  </si>
+  <si>
+    <t>Short-Haul, Europe</t>
+  </si>
+  <si>
+    <t>Paris, Amsterdam, Frankfurt, Madrid, Rome, Larnaca</t>
+  </si>
+  <si>
+    <t>Long-Haul, North America</t>
+  </si>
+  <si>
+    <t>New York JFK, Los Angeles, Chicago, Toronto, San Francisco</t>
+  </si>
+  <si>
+    <t>Long-Haul, Middle East</t>
+  </si>
+  <si>
+    <t>Dubai, Doha, Abu Dhabi, Bahrain</t>
+  </si>
+  <si>
+    <t>Long-Haul, Asia</t>
+  </si>
+  <si>
+    <t>Singapore, Tokyo, Hong Kong, Bangkok, Delhi</t>
+  </si>
+  <si>
+    <t>Lounge Eligibility Lookup Table</t>
+  </si>
+  <si>
+    <t>Question</t>
+  </si>
+  <si>
+    <t>Response</t>
+  </si>
+  <si>
+    <t>1. How did you choose to group the flights?</t>
+  </si>
+  <si>
+    <t>I grouped flights by haul (Short-Haul vs Long-Haul) and destination region (Europe, North America, Middle East, Asia). This captures structural differences in aircraft configuration and passenger mix. Short-haul flights have smaller aircraft with no first class, while long-haul flights have larger aircraft with first, business, and economy cabins, which directly impacts lounge eligibility percentages.</t>
+  </si>
+  <si>
+    <t>2. Why do your groupings make sense for this type of modeling?</t>
+  </si>
+  <si>
+    <t>The groupings use stable characteristics of BA route network (haul and region) rather than flight-specific details. Haul drives aircraft type and seat configuration; region reflects demand patterns. These categories are easy to apply to future schedules because BA knows its route network in advance, so flights can always be classified into these groups without exact aircraft or flight number details.</t>
+  </si>
+  <si>
+    <t>3. What assumptions did you make and what is the reasoning behind them?</t>
+  </si>
+  <si>
+    <t>Assumptions: (1) Tier 1 (Concorde Room) is 0.2-0.3% of passengers - driven by top-tier loyalty status holders, relatively rare. (2) Tier 2 (First Lounge) is 2.5-4.5% - higher on short-haul due to more Silver cardholders. (3) Tier 3 (Club Lounge) is 10-17% - higher on short-haul where Club Europe has a larger share of the smaller cabin. These are based on average tier eligibility counts from the sample flight schedule data, rounded to clean figures for future applicability.</t>
+  </si>
+  <si>
+    <t>4. How can your model scale to future or unknown schedules?</t>
+  </si>
+  <si>
+    <t>The lookup table is inherently scalable because it uses broad categories (haul + region) rather than specific flights or aircraft types. As BA adds or removes routes, each new flight can be classified into existing groups based on destination region. If BA introduces new regions or configurations, a new row can be added using the same methodology. The percentage estimates can also be refined over time as more data becomes available.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.0"/>
+  </numFmts>
   <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -255,7 +312,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -264,7 +321,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="49" fontId="3" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="3" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -280,6 +337,9 @@
     <xf numFmtId="49" fontId="5" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="4" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -701,24 +761,24 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="D8:I24"/>
-  <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="4" max="4" width="28.453125" customWidth="1"/>
-    <col min="5" max="5" width="31.58984375" customWidth="1"/>
+    <col min="5" max="5" width="31.54296875" customWidth="1"/>
     <col min="6" max="6" width="16.81640625" customWidth="1"/>
     <col min="7" max="7" width="16.453125" customWidth="1"/>
     <col min="8" max="8" width="15.453125" customWidth="1"/>
-    <col min="9" max="9" width="38.76953125" customWidth="1"/>
-    <col min="10" max="10" width="9.1328125" customWidth="1"/>
+    <col min="9" max="9" width="38.7265625" customWidth="1"/>
+    <col min="10" max="10" width="9.08984375" customWidth="1"/>
     <col min="12" max="12" width="26.90625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="8" spans="4:9" ht="23" x14ac:dyDescent="1">
+    <row r="8" spans="4:9" ht="23" x14ac:dyDescent="0.5">
       <c r="D8" s="1" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="10" spans="4:9" ht="18" x14ac:dyDescent="0.75">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="10" spans="4:9" ht="18" x14ac:dyDescent="0.35">
       <c r="D10" s="2" t="s">
         <v>0</v>
       </c>
@@ -738,39 +798,79 @@
         <v>5</v>
       </c>
     </row>
-    <row r="11" spans="4:9" ht="20.25" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="D11" s="3"/>
-      <c r="E11" s="3"/>
-      <c r="F11" s="3"/>
-      <c r="G11" s="3"/>
-      <c r="H11" s="3"/>
+    <row r="11" spans="4:9" ht="20.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="D11" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="F11" s="14">
+        <v>0.3</v>
+      </c>
+      <c r="G11" s="14">
+        <v>4.5</v>
+      </c>
+      <c r="H11" s="14">
+        <v>17</v>
+      </c>
       <c r="I11" s="3"/>
     </row>
-    <row r="12" spans="4:9" ht="20.5" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="D12" s="4"/>
-      <c r="E12" s="4"/>
-      <c r="F12" s="4"/>
-      <c r="G12" s="4"/>
-      <c r="H12" s="4"/>
+    <row r="12" spans="4:9" ht="20.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="D12" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="E12" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="F12" s="15">
+        <v>0.2</v>
+      </c>
+      <c r="G12" s="15">
+        <v>3</v>
+      </c>
+      <c r="H12" s="15">
+        <v>10.5</v>
+      </c>
       <c r="I12" s="4"/>
     </row>
-    <row r="13" spans="4:9" ht="20.75" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="D13" s="3"/>
-      <c r="E13" s="3"/>
-      <c r="F13" s="3"/>
-      <c r="G13" s="3"/>
-      <c r="H13" s="3"/>
+    <row r="13" spans="4:9" ht="20.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="D13" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E13" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F13" s="14">
+        <v>0.2</v>
+      </c>
+      <c r="G13" s="14">
+        <v>3</v>
+      </c>
+      <c r="H13" s="14">
+        <v>10.5</v>
+      </c>
       <c r="I13" s="3"/>
     </row>
-    <row r="14" spans="4:9" ht="20.75" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="D14" s="5"/>
-      <c r="E14" s="5"/>
-      <c r="F14" s="5"/>
-      <c r="G14" s="5"/>
-      <c r="H14" s="5"/>
+    <row r="14" spans="4:9" ht="20.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="D14" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="E14" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="F14" s="16">
+        <v>0.2</v>
+      </c>
+      <c r="G14" s="16">
+        <v>2.5</v>
+      </c>
+      <c r="H14" s="16">
+        <v>10</v>
+      </c>
       <c r="I14" s="5"/>
     </row>
-    <row r="15" spans="4:9" ht="20.25" customHeight="1" x14ac:dyDescent="0.75">
+    <row r="15" spans="4:9" ht="20.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="D15" s="3"/>
       <c r="E15" s="3"/>
       <c r="F15" s="3"/>
@@ -778,7 +878,7 @@
       <c r="H15" s="3"/>
       <c r="I15" s="3"/>
     </row>
-    <row r="16" spans="4:9" ht="20.5" customHeight="1" x14ac:dyDescent="0.75">
+    <row r="16" spans="4:9" ht="20.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="D16" s="4"/>
       <c r="E16" s="4"/>
       <c r="F16" s="4"/>
@@ -786,7 +886,7 @@
       <c r="H16" s="4"/>
       <c r="I16" s="4"/>
     </row>
-    <row r="17" spans="4:9" ht="20.75" customHeight="1" x14ac:dyDescent="0.75">
+    <row r="17" spans="4:9" ht="20.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="D17" s="3"/>
       <c r="E17" s="3"/>
       <c r="F17" s="3"/>
@@ -794,7 +894,7 @@
       <c r="H17" s="3"/>
       <c r="I17" s="3"/>
     </row>
-    <row r="18" spans="4:9" ht="20.5" customHeight="1" x14ac:dyDescent="0.75">
+    <row r="18" spans="4:9" ht="20.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="D18" s="4"/>
       <c r="E18" s="4"/>
       <c r="F18" s="4"/>
@@ -802,7 +902,7 @@
       <c r="H18" s="4"/>
       <c r="I18" s="4"/>
     </row>
-    <row r="19" spans="4:9" ht="20.75" customHeight="1" x14ac:dyDescent="0.75">
+    <row r="19" spans="4:9" ht="20.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="D19" s="3"/>
       <c r="E19" s="3"/>
       <c r="F19" s="3"/>
@@ -810,7 +910,7 @@
       <c r="H19" s="3"/>
       <c r="I19" s="3"/>
     </row>
-    <row r="20" spans="4:9" ht="20.75" customHeight="1" x14ac:dyDescent="0.75">
+    <row r="20" spans="4:9" ht="20.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="D20" s="6"/>
       <c r="E20" s="6"/>
       <c r="F20" s="6"/>
@@ -818,7 +918,7 @@
       <c r="H20" s="6"/>
       <c r="I20" s="6"/>
     </row>
-    <row r="21" spans="4:9" ht="20.75" customHeight="1" x14ac:dyDescent="0.75">
+    <row r="21" spans="4:9" ht="20.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="D21" s="6"/>
       <c r="E21" s="6"/>
       <c r="F21" s="6"/>
@@ -826,8 +926,8 @@
       <c r="H21" s="6"/>
       <c r="I21" s="6"/>
     </row>
-    <row r="23" spans="4:9" ht="21.5" customHeight="1" x14ac:dyDescent="0.75"/>
-    <row r="24" spans="4:9" ht="55" customHeight="1" x14ac:dyDescent="0.75"/>
+    <row r="23" spans="4:9" ht="21.5" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="24" spans="4:9" ht="55" customHeight="1" x14ac:dyDescent="0.35"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -836,49 +936,89 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3D51397D-80FE-4B58-8712-003CA23A8E8E}">
-  <dimension ref="A10:D15"/>
-  <sheetFormatPr defaultColWidth="167.76953125" defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
+  <dimension ref="A1:D15"/>
+  <sheetFormatPr defaultColWidth="167.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="0.54296875" customWidth="1"/>
     <col min="2" max="2" width="32.54296875" customWidth="1"/>
-    <col min="3" max="3" width="69.6796875" customWidth="1"/>
+    <col min="3" max="3" width="69.6328125" customWidth="1"/>
     <col min="4" max="4" width="75.54296875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="10" spans="3:4" ht="21.25" thickBot="1" x14ac:dyDescent="1.05">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>24</v>
+      </c>
+      <c r="B3" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>26</v>
+      </c>
+      <c r="B5" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>28</v>
+      </c>
+      <c r="B7" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>30</v>
+      </c>
+      <c r="B9" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" ht="20.5" thickBot="1" x14ac:dyDescent="0.45">
       <c r="C10" s="9" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="11" spans="3:4" ht="25" customHeight="1" x14ac:dyDescent="0.8">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.4">
       <c r="C11" s="10" t="s">
+        <v>6</v>
+      </c>
+      <c r="D11" s="11" t="s">
         <v>7</v>
       </c>
-      <c r="D11" s="11" t="s">
+    </row>
+    <row r="12" spans="1:4" ht="30.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="C12" s="12" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="12" spans="3:4" ht="30.75" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="C12" s="12" t="s">
+      <c r="D12" s="7"/>
+    </row>
+    <row r="13" spans="1:4" ht="31" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="C13" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="D12" s="7"/>
-    </row>
-    <row r="13" spans="3:4" ht="31" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="C13" s="12" t="s">
+      <c r="D13" s="7"/>
+    </row>
+    <row r="14" spans="1:4" ht="30.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="C14" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="D13" s="7"/>
-    </row>
-    <row r="14" spans="3:4" ht="30.75" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="C14" s="12" t="s">
+      <c r="D14" s="7"/>
+    </row>
+    <row r="15" spans="1:4" ht="32.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="C15" s="13" t="s">
         <v>11</v>
-      </c>
-      <c r="D14" s="7"/>
-    </row>
-    <row r="15" spans="3:4" ht="32.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.9">
-      <c r="C15" s="13" t="s">
-        <v>12</v>
       </c>
       <c r="D15" s="8"/>
     </row>

</xml_diff>